<commit_message>
Árak és eszközök változtatása
Eszközök számának megváltoztatása, új eszközök hozzáadása a listához.
</commit_message>
<xml_diff>
--- a/Javított ár tervezet.xlsx
+++ b/Javított ár tervezet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/534523f344482c23/Asztali gép/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\folla\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="168" documentId="8_{654AC442-3CCD-49B0-97CC-FE68C406ACC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25A5EFFE-62DD-44FB-A849-C04A04781A7F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE2A6268-C495-4653-A1F5-D59CBE9A28C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{9A4E7F6D-FF73-4FBA-8320-FC974226BA90}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9A4E7F6D-FF73-4FBA-8320-FC974226BA90}"/>
   </bookViews>
   <sheets>
     <sheet name="Munka1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
   <si>
     <t>NÉV</t>
   </si>
@@ -204,6 +204,9 @@
   </si>
   <si>
     <t>500M</t>
+  </si>
+  <si>
+    <t>Tablet</t>
   </si>
 </sst>
 </file>
@@ -273,7 +276,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="28">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -656,6 +659,15 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -663,7 +675,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -729,6 +741,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -745,10 +760,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1116,21 +1127,21 @@
         <v>1</v>
       </c>
       <c r="C2" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
       </c>
       <c r="E2" s="10">
         <f>B2+C2+D2</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" s="39">
         <v>40</v>
       </c>
       <c r="G2" s="7">
         <f>E2*F2</f>
-        <v>120</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -1141,21 +1152,21 @@
         <v>3</v>
       </c>
       <c r="C3" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" s="11">
         <f>B3+C3+D3</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F3" s="8">
         <v>315</v>
       </c>
       <c r="G3" s="8">
         <f t="shared" ref="G3:G6" si="0">E3*F3</f>
-        <v>3780</v>
+        <v>4410</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1169,18 +1180,18 @@
         <v>1</v>
       </c>
       <c r="D4" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="11">
         <f t="shared" ref="E4:E6" si="1">B4+C4+D4</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4" s="8">
         <v>3075</v>
       </c>
       <c r="G4" s="8">
         <f t="shared" si="0"/>
-        <v>9225</v>
+        <v>12300</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1191,10 +1202,10 @@
         <v>2</v>
       </c>
       <c r="C5" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="11">
         <f t="shared" si="1"/>
@@ -1252,21 +1263,21 @@
         <v>4</v>
       </c>
       <c r="C7" s="4">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4">
         <v>7</v>
       </c>
-      <c r="D7" s="4">
-        <v>4</v>
-      </c>
       <c r="E7" s="11">
-        <f t="shared" ref="E7:E11" si="2">B7+C7+D7</f>
-        <v>15</v>
+        <f t="shared" ref="E7:E8" si="2">B7+C7+D7</f>
+        <v>11</v>
       </c>
       <c r="F7" s="8">
         <v>1050</v>
       </c>
       <c r="G7" s="8">
-        <f t="shared" ref="G7:G16" si="3">E7*F7</f>
-        <v>15750</v>
+        <f t="shared" ref="G7:G8" si="3">E7*F7</f>
+        <v>11550</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>33</v>
@@ -1284,21 +1295,21 @@
         <v>14</v>
       </c>
       <c r="C8" s="4">
+        <v>12</v>
+      </c>
+      <c r="D8" s="4">
         <v>11</v>
-      </c>
-      <c r="D8" s="4">
-        <v>10</v>
       </c>
       <c r="E8" s="11">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F8" s="8">
         <v>1570</v>
       </c>
       <c r="G8" s="8">
         <f t="shared" si="3"/>
-        <v>54950</v>
+        <v>58090</v>
       </c>
       <c r="J8" s="3" t="s">
         <v>34</v>
@@ -1309,8 +1320,8 @@
       <c r="L8" s="15"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>11</v>
+      <c r="A9" s="47" t="s">
+        <v>42</v>
       </c>
       <c r="B9" s="4">
         <v>0</v>
@@ -1319,18 +1330,16 @@
         <v>0</v>
       </c>
       <c r="D9" s="4">
-        <v>3</v>
-      </c>
-      <c r="E9" s="11">
-        <f t="shared" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="F9" s="8">
-        <v>750</v>
-      </c>
-      <c r="G9" s="8">
-        <f t="shared" si="3"/>
-        <v>2250</v>
+        <v>2</v>
+      </c>
+      <c r="E9" s="29">
+        <v>2</v>
+      </c>
+      <c r="F9" s="45">
+        <v>500</v>
+      </c>
+      <c r="G9" s="46">
+        <v>1000</v>
       </c>
       <c r="J9" s="3"/>
       <c r="K9" s="29"/>
@@ -1338,27 +1347,27 @@
     </row>
     <row r="10" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" s="4">
         <v>0</v>
       </c>
       <c r="D10" s="4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E10" s="11">
         <f>B10+C10+D10</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="8">
-        <v>52680</v>
+        <v>750</v>
       </c>
       <c r="G10" s="8">
-        <f t="shared" si="3"/>
-        <v>52680</v>
+        <f>E10*F10</f>
+        <v>1500</v>
       </c>
       <c r="J10" s="32" t="s">
         <v>38</v>
@@ -1374,40 +1383,40 @@
         <v>12</v>
       </c>
       <c r="B11" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C11" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="4">
         <v>0</v>
       </c>
       <c r="E11" s="11">
-        <f t="shared" si="2"/>
+        <f>B11+C11+D11</f>
         <v>1</v>
       </c>
       <c r="F11" s="8">
         <v>52680</v>
       </c>
       <c r="G11" s="8">
-        <f t="shared" si="3"/>
+        <f>E11*F11</f>
         <v>52680</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="B12" s="4">
         <v>0</v>
       </c>
       <c r="C12" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" s="4">
-        <v>1</v>
-      </c>
-      <c r="E12" s="17">
+        <v>0</v>
+      </c>
+      <c r="E12" s="11">
         <f>B12+C12+D12</f>
         <v>1</v>
       </c>
@@ -1415,153 +1424,155 @@
         <v>52680</v>
       </c>
       <c r="G12" s="8">
-        <f t="shared" si="3"/>
+        <f>E12*F12</f>
         <v>52680</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="B13" s="4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C13" s="4">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D13" s="4">
-        <v>2</v>
-      </c>
-      <c r="E13" s="11">
+        <v>1</v>
+      </c>
+      <c r="E13" s="17">
         <f>B13+C13+D13</f>
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="F13" s="8">
-        <v>510</v>
+        <v>52680</v>
       </c>
       <c r="G13" s="8">
-        <f t="shared" si="3"/>
-        <v>5610</v>
+        <f>E13*F13</f>
+        <v>52680</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C14" s="4">
+        <v>6</v>
+      </c>
+      <c r="D14" s="4">
         <v>2</v>
-      </c>
-      <c r="D14" s="4">
-        <v>1</v>
       </c>
       <c r="E14" s="11">
         <f>B14+C14+D14</f>
-        <v>3</v>
-      </c>
-      <c r="F14" s="18">
-        <v>369</v>
+        <v>11</v>
+      </c>
+      <c r="F14" s="8">
+        <v>510</v>
       </c>
       <c r="G14" s="8">
-        <f t="shared" si="3"/>
-        <v>1107</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
-        <v>15</v>
+        <f>E14*F14</f>
+        <v>5610</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="B15" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" s="4">
         <v>2</v>
       </c>
       <c r="D15" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="11">
         <f>B15+C15+D15</f>
         <v>3</v>
       </c>
-      <c r="F15" s="8">
-        <v>2500</v>
+      <c r="F15" s="18">
+        <v>369</v>
       </c>
       <c r="G15" s="8">
-        <f t="shared" si="3"/>
-        <v>7500</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
-        <v>16</v>
+        <f>E15*F15</f>
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="B16" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C16" s="4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D16" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" s="11">
         <f>B16+C16+D16</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F16" s="8">
-        <v>650</v>
+        <v>2500</v>
       </c>
       <c r="G16" s="8">
-        <f t="shared" si="3"/>
-        <v>650</v>
+        <f>E16*F16</f>
+        <v>7500</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="F17" s="6">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4">
+        <v>0</v>
+      </c>
+      <c r="C17" s="4">
+        <v>1</v>
+      </c>
+      <c r="D17" s="4">
+        <v>1</v>
+      </c>
+      <c r="E17" s="11">
+        <f>B17+C17+D17</f>
         <v>2</v>
       </c>
-      <c r="G17" s="14">
-        <v>3000</v>
+      <c r="F17" s="8">
+        <v>650</v>
+      </c>
+      <c r="G17" s="8">
+        <f>E17*F17</f>
+        <v>1300</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="14.4" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18" s="16" t="s">
-        <v>41</v>
+        <v>24</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>20</v>
       </c>
       <c r="F18" s="6">
-        <v>6</v>
-      </c>
-      <c r="G18" s="8">
+        <v>2</v>
+      </c>
+      <c r="G18" s="14">
         <v>3000</v>
       </c>
       <c r="J18" s="43" t="s">
@@ -1569,50 +1580,72 @@
       </c>
       <c r="K18" s="44"/>
       <c r="L18" s="33">
-        <f>G2+G3+G4+G5+G7+G8+G9+G10+G11+G12+G13+G14+G15+G16+G17+G18+G19+G20+K10+G6</f>
-        <v>330427</v>
+        <f>G2+G3+G4+G5+G7+G8+G10+G11+G12+G13+G14+G15+G16+G17+G18+G19+G20+G21+K10+G6+G9</f>
+        <v>333932</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="F19" s="6">
+        <v>6</v>
+      </c>
+      <c r="G19" s="8">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A20" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B20" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20" t="s">
+      <c r="C20" s="20"/>
+      <c r="D20" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="21" t="s">
+      <c r="E20" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="F19" s="22">
+      <c r="F20" s="22">
         <v>17</v>
       </c>
-      <c r="G19" s="23">
+      <c r="G20" s="23">
         <v>3400</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="24" t="s">
+    <row r="21" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="40"/>
-      <c r="C20" s="40"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="26" t="s">
+      <c r="B21" s="40"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F20" s="27">
+      <c r="F21" s="27">
         <v>2634</v>
       </c>
-      <c r="G20" s="28">
+      <c r="G21" s="28">
         <v>31608</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="I22" s="9"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">

</xml_diff>